<commit_message>
Round 3 corrections on Guide
</commit_message>
<xml_diff>
--- a/guide/syntropy-guide-cms-template.xlsx
+++ b/guide/syntropy-guide-cms-template.xlsx
@@ -303,39 +303,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>